<commit_message>
just need to automate script
</commit_message>
<xml_diff>
--- a/lw3Tweets.xlsx
+++ b/lw3Tweets.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Date Created</t>
   </si>
@@ -28,27 +28,54 @@
     <t>DaysOfCoding</t>
   </si>
   <si>
-    <t>(2022, 12, 30)</t>
+    <t>(2023, 1, 1)</t>
+  </si>
+  <si>
+    <t>(2022, 12, 31)</t>
+  </si>
+  <si>
+    <t>heheh</t>
+  </si>
+  <si>
+    <t>TiwariAnkitb</t>
+  </si>
+  <si>
+    <t>rahul3526</t>
   </si>
   <si>
     <t>PandeyAshwini9</t>
   </si>
   <si>
-    <t>TiwariAnkitb</t>
-  </si>
-  <si>
-    <t>Day 44 of #100DaysOfCode with @TiwariAnkitb by @LearnWeb3DAO .
-Build your own fully on-chain DAO to invest in NFTs✅
-check it...
-https://t.co/HgLNVUNvp7
-#Web3 
-#web3community https://t.co/R0fJjQ9caG</t>
-  </si>
-  <si>
-    <t>Day 45 of #100DaysOfCode with @PandeyAshwini9 from @LearnWeb3DAO.
-Completed 85% on the sophomore level and achieving more...
-#Web3 
-#web3community</t>
+    <t>Day 47 of #100DaysOfCode with @TiwariAnkitb from @LearnWeb3DAO.
+In progress....
+Build your own Decentraized exchange like Uniswap.
+Solidity code ✅
+Ether.js✅
+Hardhat ✅
+NextJs❌
+Excited for tomorrow...
+#Web3
+#Blockchain
+#100daysofcodingchallenge</t>
+  </si>
+  <si>
+    <t>Day 47 of #100DaysOfCode with @PandeyAshwini9 from @LearnWeb3DAO.
+In progress....
+Build your own Decentraized exchange like Uniswap.
+Solidity code ✅
+Ether.js✅
+Hardhat ✅
+NextJs❌
+Excited for tomorrow...
+#Web3
+#Blockchain
+#100daysofcodingchallenge</t>
+  </si>
+  <si>
+    <t>Round 2.
+Day 10 of #100DaysOfCode .
+Made a video on How to get started with rainbow kit. Also gave a easy solution to the hydration error problem Had been facing it for so long. Check out the video in comments below. I would like to thank @LearnWeb3DAO  
+https://t.co/rQ2h5tDpsQ</t>
   </si>
 </sst>
 </file>
@@ -406,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -428,13 +455,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -442,12 +469,40 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="D3">
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added links to spreadsheet
</commit_message>
<xml_diff>
--- a/lw3Tweets.xlsx
+++ b/lw3Tweets.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Date Created</t>
   </si>
@@ -25,64 +25,86 @@
     <t>Tweets</t>
   </si>
   <si>
+    <t>Link</t>
+  </si>
+  <si>
     <t>DaysOfCoding</t>
   </si>
   <si>
-    <t>(2023, 1, 1)</t>
-  </si>
-  <si>
-    <t>(2022, 12, 31)</t>
-  </si>
-  <si>
-    <t>heheh</t>
-  </si>
-  <si>
-    <t>TiwariAnkitb</t>
-  </si>
-  <si>
-    <t>rahul3526</t>
-  </si>
-  <si>
-    <t>PandeyAshwini9</t>
-  </si>
-  <si>
-    <t>Day 47 of #100DaysOfCode with @TiwariAnkitb from @LearnWeb3DAO.
-In progress....
-Build your own Decentraized exchange like Uniswap.
-Solidity code ✅
-Ether.js✅
-Hardhat ✅
-NextJs❌
-Excited for tomorrow...
-#Web3
-#Blockchain
-#100daysofcodingchallenge</t>
-  </si>
-  <si>
-    <t>Day 47 of #100DaysOfCode with @PandeyAshwini9 from @LearnWeb3DAO.
-In progress....
-Build your own Decentraized exchange like Uniswap.
-Solidity code ✅
-Ether.js✅
-Hardhat ✅
-NextJs❌
-Excited for tomorrow...
-#Web3
-#Blockchain
-#100daysofcodingchallenge</t>
-  </si>
-  <si>
-    <t>Round 2.
-Day 10 of #100DaysOfCode .
-Made a video on How to get started with rainbow kit. Also gave a easy solution to the hydration error problem Had been facing it for so long. Check out the video in comments below. I would like to thank @LearnWeb3DAO  
-https://t.co/rQ2h5tDpsQ</t>
+    <t>(2023, 1, 5)</t>
+  </si>
+  <si>
+    <t>Syvelline</t>
+  </si>
+  <si>
+    <t>0xCylax</t>
+  </si>
+  <si>
+    <t>ArshiaZojaji</t>
+  </si>
+  <si>
+    <t>yc_crypto</t>
+  </si>
+  <si>
+    <t>cjski_web3</t>
+  </si>
+  <si>
+    <t>Day- 38 of #100DaysOfCode 
+✅Spent reading about Ethereum and Bitcoin in-depth and continued freshman track @LearnWeb3DAO 
+✅Completed lesson 1 of solidity @CryptoZombiesHQ 
+Most productive day of a challenge since I picked it again
+#100daysofcodechallenge #100daysofcoding https://t.co/seWOV7BYgr</t>
+  </si>
+  <si>
+    <t>Day 18 of #100DaysOfCode
+- solved few problems using linear search algorithm
+- almost completed building shopping app project using React
+- learned more about hardhat on @AlchemyLearn (60% of week 4 ✅)
+- completed 30% of sophomore track🏕 on @LearnWeb3DAO https://t.co/5lShrbLEy5</t>
+  </si>
+  <si>
+    <t>Day 4⃣ of journey to learn #smartcontracts 🥳
+I'm joining the #100daysofcode challenge with the @LearnWeb3DAO community! 💻
+We'll be focusing on Web3 development for 100 days!
+Join us here👇
+🔗https://t.co/hoEtohzV5Z
+#100DaysofCodeLW3 https://t.co/8vBrLGM7iI</t>
+  </si>
+  <si>
+    <t>Planning to start #100daysofcode once again. will document my journey here and @LearnWeb3DAO and @scdevstr discord channels. 
+I will plan my calendar this weekend and starting on monday.
+#100DAYSOFCODELW3</t>
+  </si>
+  <si>
+    <t>Alright champs, here's what we are going to do together as web3 community 😎
+As it was officially announced in @LearnWeb3DAO discord, on 9th of January we are going to start community driven #100DaysOfCode challenge. 
+@haardikkk
+@Haezurath
+@KhanAbbas201
+@LarryCutts6
+👇</t>
+  </si>
+  <si>
+    <t>https://twitter.com/Syvelline/status/1611059503746928640</t>
+  </si>
+  <si>
+    <t>https://twitter.com/0xCylax/status/1611030272782499840</t>
+  </si>
+  <si>
+    <t>https://twitter.com/ArshiaZojaji/status/1611032640710389760</t>
+  </si>
+  <si>
+    <t>https://twitter.com/yc_crypto/status/1610929639576293376</t>
+  </si>
+  <si>
+    <t>https://twitter.com/cjski_web3/status/1610812225807056896</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +119,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -131,16 +160,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -433,10 +468,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -449,36 +484,45 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -486,27 +530,57 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="D5">
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="D3" r:id="rId2"/>
+    <hyperlink ref="D4" r:id="rId3"/>
+    <hyperlink ref="D5" r:id="rId4"/>
+    <hyperlink ref="D6" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added flask and schedule functionality
</commit_message>
<xml_diff>
--- a/lw3Tweets.xlsx
+++ b/lw3Tweets.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
   <si>
     <t>Date Created</t>
   </si>
@@ -31,22 +31,63 @@
     <t>DaysOfCoding</t>
   </si>
   <si>
+    <t>(2023, 1, 6)</t>
+  </si>
+  <si>
     <t>(2023, 1, 5)</t>
   </si>
   <si>
+    <t>(2023, 1, 7)</t>
+  </si>
+  <si>
+    <t>ArshiaZojaji</t>
+  </si>
+  <si>
+    <t>0xCylax</t>
+  </si>
+  <si>
     <t>Syvelline</t>
   </si>
   <si>
-    <t>0xCylax</t>
-  </si>
-  <si>
-    <t>ArshiaZojaji</t>
-  </si>
-  <si>
     <t>yc_crypto</t>
   </si>
   <si>
     <t>cjski_web3</t>
+  </si>
+  <si>
+    <t>web3Learning2</t>
+  </si>
+  <si>
+    <t>Maitrayeedas9</t>
+  </si>
+  <si>
+    <t>a20zCrypto</t>
+  </si>
+  <si>
+    <t>0xLesanders</t>
+  </si>
+  <si>
+    <t>rav3kid</t>
+  </si>
+  <si>
+    <t>Justacanuk81</t>
+  </si>
+  <si>
+    <t>Daily Update Tweet: 
+Day 5⃣ of #100daysofcode w/ @LearnWeb3DAO
+JavaScript are fundamentals are finished today, wow that was big. 🥳🔥
+worked on:
+1. Objects
+2. Loops
+3. Functions
+#100DaysofCodeLW3 #javascript https://t.co/qdGzkLVdMr</t>
+  </si>
+  <si>
+    <t>Day 19 of #100DaysOfCode 
+- learned about binary search algorithm 
+- learned about receive &amp;amp; revert functions, function modifiers on AU (w4 - 70%) 
+- 'working of Proof of Stake' on @LearnWeb3DAO 
+- added media queries &amp;amp; products page in shopping app project https://t.co/vfAZf7LqYL</t>
   </si>
   <si>
     <t>Day- 38 of #100DaysOfCode 
@@ -54,21 +95,6 @@
 ✅Completed lesson 1 of solidity @CryptoZombiesHQ 
 Most productive day of a challenge since I picked it again
 #100daysofcodechallenge #100daysofcoding https://t.co/seWOV7BYgr</t>
-  </si>
-  <si>
-    <t>Day 18 of #100DaysOfCode
-- solved few problems using linear search algorithm
-- almost completed building shopping app project using React
-- learned more about hardhat on @AlchemyLearn (60% of week 4 ✅)
-- completed 30% of sophomore track🏕 on @LearnWeb3DAO https://t.co/5lShrbLEy5</t>
-  </si>
-  <si>
-    <t>Day 4⃣ of journey to learn #smartcontracts 🥳
-I'm joining the #100daysofcode challenge with the @LearnWeb3DAO community! 💻
-We'll be focusing on Web3 development for 100 days!
-Join us here👇
-🔗https://t.co/hoEtohzV5Z
-#100DaysofCodeLW3 https://t.co/8vBrLGM7iI</t>
   </si>
   <si>
     <t>Planning to start #100daysofcode once again. will document my journey here and @LearnWeb3DAO and @scdevstr discord channels. 
@@ -85,19 +111,79 @@
 👇</t>
   </si>
   <si>
+    <t>I'm joining the #100daysofcode challenge with the @LearnWeb3DAO community! 💻
+We'll be focusing on Web3 development for 100 days!
+Join us here👇
+https://t.co/WmBIxayEod
+#100DaysofCodeLW3</t>
+  </si>
+  <si>
+    <t>I'm joining the #100daysofcode challenge with the @LearnWeb3DAO community! 💻
+I’ll be focusing on Web3 development for 100 days!
+Starting from January 9th.</t>
+  </si>
+  <si>
+    <t>Wanted to get an early head start...
+Day 1 of #100DaysOfCode with @LearnWeb3DAO
+-Research on effective GitHub use
+-JavaScript Rock, Paper, Scissors program focusing on different JS function syntax
+#100DaysofCodeLW3
+#Web3
+#web3community 
+@Codecademy</t>
+  </si>
+  <si>
+    <t>Day 4-5 | #100DaysOfWeb3 &amp;amp; #100DaysOfCode 
+• Finished Solidity Course 
+I will work on my final project for practicum.
+• Also will follow Freshman level on @LearnWeb3DAO https://t.co/A6aYqEjLZn</t>
+  </si>
+  <si>
+    <t>I'm joining the #100daysofcode challenge with the @LearnWeb3DAO community! 💻
+We'll be focusing on Web3 development for 100 days!
+Join us here👇
+https://t.co/SyVMQByYkK
+#100DaysofCodeLW3</t>
+  </si>
+  <si>
+    <t>I'm joining the #100daysofcode challenge with the @LearnWeb3DAO community! 💻
+We'll be focusing on Web3 development for 100 days!
+Join us here👇
+https://t.co/9epZdiLLFL
+#100DaysofCodeLW3</t>
+  </si>
+  <si>
+    <t>https://twitter.com/ArshiaZojaji/status/1611393669428350979</t>
+  </si>
+  <si>
+    <t>https://twitter.com/0xCylax/status/1611394241904926721</t>
+  </si>
+  <si>
     <t>https://twitter.com/Syvelline/status/1611059503746928640</t>
   </si>
   <si>
-    <t>https://twitter.com/0xCylax/status/1611030272782499840</t>
-  </si>
-  <si>
-    <t>https://twitter.com/ArshiaZojaji/status/1611032640710389760</t>
-  </si>
-  <si>
     <t>https://twitter.com/yc_crypto/status/1610929639576293376</t>
   </si>
   <si>
     <t>https://twitter.com/cjski_web3/status/1610812225807056896</t>
+  </si>
+  <si>
+    <t>https://twitter.com/web3Learning2/status/1611323420074975232</t>
+  </si>
+  <si>
+    <t>https://twitter.com/Maitrayeedas9/status/1611314578625028096</t>
+  </si>
+  <si>
+    <t>https://twitter.com/a20zCrypto/status/1611478248202047488</t>
+  </si>
+  <si>
+    <t>https://twitter.com/0xLesanders/status/1611705616476831744</t>
+  </si>
+  <si>
+    <t>https://twitter.com/rav3kid/status/1611626477900165123</t>
+  </si>
+  <si>
+    <t>https://twitter.com/Justacanuk81/status/1611756569502552070</t>
   </si>
 </sst>
 </file>
@@ -468,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -493,16 +579,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -510,30 +596,30 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -541,16 +627,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -558,18 +644,120 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6">
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12">
         <v>1</v>
       </c>
     </row>
@@ -580,6 +768,12 @@
     <hyperlink ref="D4" r:id="rId3"/>
     <hyperlink ref="D5" r:id="rId4"/>
     <hyperlink ref="D6" r:id="rId5"/>
+    <hyperlink ref="D7" r:id="rId6"/>
+    <hyperlink ref="D8" r:id="rId7"/>
+    <hyperlink ref="D9" r:id="rId8"/>
+    <hyperlink ref="D10" r:id="rId9"/>
+    <hyperlink ref="D11" r:id="rId10"/>
+    <hyperlink ref="D12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>